<commit_message>
Product #13 Video V3.1 FINAL: no internal labels, privacy-safe IDs
- Remove the DRAFT/RECONSTRUCTION footer via an explicit, recorded
  provenance.listing_approval (owner, date, note); dummy sources can
  never be approved.
- P13 workbook: STU-001..STU-006 replace name-style student labels;
  Dashboard + Progress Log re-captured (geometry and values unchanged,
  still verified against recalculated cells).
- Re-centre the scene-2 ring on the new Progress Log row.
- QA: OCR every key frame for internal labels; privacy checks (no
  person-name patterns in workbook data or frames, safe ID format,
  IDs visible); fix stale key-frame reuse on the last frame.
- V3.1 QA: PASS, 100 pass / 0 warn / 0 fail.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Je8YSkF1eYHDKU2du3MKbu
</commit_message>
<xml_diff>
--- a/video-engine/sources/p13-iep-tracker/workbook/p13_reconstruction_after.xlsx
+++ b/video-engine/sources/p13-iep-tracker/workbook/p13_reconstruction_after.xlsx
@@ -782,7 +782,7 @@
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Ava M.</t>
+          <t>STU-001</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>Liam R.</t>
+          <t>STU-002</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Noah K.</t>
+          <t>STU-003</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>Mia T.</t>
+          <t>STU-004</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>Ella J.</t>
+          <t>STU-005</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>Lucas P.</t>
+          <t>STU-006</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="B5" s="21" t="inlineStr">
         <is>
-          <t>Ava M.</t>
+          <t>STU-001</t>
         </is>
       </c>
       <c r="C5" s="21" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="B6" s="21" t="inlineStr">
         <is>
-          <t>Ava M.</t>
+          <t>STU-001</t>
         </is>
       </c>
       <c r="C6" s="21" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="B7" s="21" t="inlineStr">
         <is>
-          <t>Liam R.</t>
+          <t>STU-002</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B8" s="21" t="inlineStr">
         <is>
-          <t>Liam R.</t>
+          <t>STU-002</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>Noah K.</t>
+          <t>STU-003</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>Noah K.</t>
+          <t>STU-003</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Mia T.</t>
+          <t>STU-004</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>Mia T.</t>
+          <t>STU-004</t>
         </is>
       </c>
       <c r="C12" s="21" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>Ella J.</t>
+          <t>STU-005</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>Ella J.</t>
+          <t>STU-005</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>Lucas P.</t>
+          <t>STU-006</t>
         </is>
       </c>
       <c r="C15" s="21" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>Lucas P.</t>
+          <t>STU-006</t>
         </is>
       </c>
       <c r="C16" s="21" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>Mia T.</t>
+          <t>STU-004</t>
         </is>
       </c>
       <c r="C17" s="21" t="inlineStr">

</xml_diff>